<commit_message>
Add Annual Tax Management, precomputed data packages, and Annual Leadership Report
</commit_message>
<xml_diff>
--- a/03_DAU_RA/Bao_Cao_Kiem_Do_Thue_TNCN_Thang_09_2026.xlsx
+++ b/03_DAU_RA/Bao_Cao_Kiem_Do_Thue_TNCN_Thang_09_2026.xlsx
@@ -618,7 +618,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Ngày xuất báo cáo: 14/10/2026 09:07:53</t>
+          <t>Ngày xuất báo cáo: 14/10/2026 09:27:06</t>
         </is>
       </c>
     </row>
@@ -34165,7 +34165,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Ngày xuất báo cáo: 14/10/2026 09:07:54</t>
+          <t>Ngày xuất báo cáo: 14/10/2026 09:27:07</t>
         </is>
       </c>
     </row>
@@ -54462,7 +54462,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Ngày xuất báo cáo: 14/10/2026 09:07:54</t>
+          <t>Ngày xuất báo cáo: 14/10/2026 09:27:07</t>
         </is>
       </c>
     </row>
@@ -66411,7 +66411,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Ngày xuất báo cáo: 14/10/2026 09:07:54</t>
+          <t>Ngày xuất báo cáo: 14/10/2026 09:27:07</t>
         </is>
       </c>
     </row>

</xml_diff>